<commit_message>
Complete OffenderWatch QA assignment
</commit_message>
<xml_diff>
--- a/docs/test-cases/OffenderWatch_Test_Suite.xlsx
+++ b/docs/test-cases/OffenderWatch_Test_Suite.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\noamh\Desktop\offenderwatch-qa-assignment\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\noamh\Desktop\offenderwatch-qa-assignment\offenderwatch-qa-assignment\docs\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCEC8860-876F-4360-91F9-C0DB9A99613E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05C2482A-5335-4068-B381-FB961D196344}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{FB3FEA46-C9C7-4B84-9C3C-89481DF81E28}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="368">
   <si>
     <t xml:space="preserve">test ID </t>
   </si>
@@ -64,9 +64,6 @@
   </si>
   <si>
     <t>UI</t>
-  </si>
-  <si>
-    <t>Not Run</t>
   </si>
   <si>
     <t>-</t>
@@ -352,18 +349,6 @@
     <t>FR-03, FR-04</t>
   </si>
   <si>
-    <t>Verify future date of birth is rejected when editing an offender</t>
-  </si>
-  <si>
-    <t>An existing offender with a valid Date of Birth is available.</t>
-  </si>
-  <si>
-    <t>1. Record the offender's current Date of Birth. 2. Open the offender's edit form. 3. Replace the Date of Birth with a future date. 4. Attempt to save the changes. 5. Reopen the offender.</t>
-  </si>
-  <si>
-    <t>The update is rejected with a clear error message. The offender retains the previous valid Date of Birth and the invalid change is not persisted.</t>
-  </si>
-  <si>
     <t>Verify offender deletion can be cancelled from the confirmation prompt</t>
   </si>
   <si>
@@ -439,9 +424,6 @@
     <t>The UI displays the same Date of Birth returned by the API, formatted as DD/MM/YYYY.</t>
   </si>
   <si>
-    <t>1. Retrieve the test offender created in UI-009 through the API. 2.Record the stored Date of Birth returned by the API. 3.Open the same offender in the UI. 4.Compare the displayed Date of Birth with the API value</t>
-  </si>
-  <si>
     <t>UI-022</t>
   </si>
   <si>
@@ -559,9 +541,6 @@
     <t>Add Location form is available.</t>
   </si>
   <si>
-    <t>1. Enter otherwise valid location data. 2. Enter an invalid latitude or longitude value outside the valid coordinate range. 3. Attempt to save.</t>
-  </si>
-  <si>
     <t>The invalid location point is rejected and is not saved.</t>
   </si>
   <si>
@@ -571,27 +550,18 @@
     <t>Verify negative speed is rejected</t>
   </si>
   <si>
-    <t>1. Enter otherwise valid location data. 2. Enter a speed value below 0. 3. Attempt to save.</t>
-  </si>
-  <si>
     <t>The submission is rejected and the location point is not saved.</t>
   </si>
   <si>
     <t>Verify battery value must be between 0 and 100</t>
   </si>
   <si>
-    <t>1. Enter otherwise valid location data with battery below 0 and attempt to save. 2. Repeat with battery above 100.</t>
-  </si>
-  <si>
     <t>Both invalid submissions are rejected and no location point is saved.</t>
   </si>
   <si>
     <t>Verify signal value must be between 1 and 5</t>
   </si>
   <si>
-    <t>1. Enter otherwise valid location data with signal below 1 and attempt to save. 2. Repeat with signal above 5.</t>
-  </si>
-  <si>
     <t>Verify Latest Reading updates after adding the most recent location point</t>
   </si>
   <si>
@@ -712,9 +682,6 @@
     <t>UI-040</t>
   </si>
   <si>
-    <t>API-001</t>
-  </si>
-  <si>
     <t>API-01</t>
   </si>
   <si>
@@ -1946,36 +1913,6 @@
     </r>
   </si>
   <si>
-    <t>API-006</t>
-  </si>
-  <si>
-    <t>API-002</t>
-  </si>
-  <si>
-    <t>API-003</t>
-  </si>
-  <si>
-    <t>API-004</t>
-  </si>
-  <si>
-    <t>API-005</t>
-  </si>
-  <si>
-    <t>API-007</t>
-  </si>
-  <si>
-    <t>API-008</t>
-  </si>
-  <si>
-    <t>API-009</t>
-  </si>
-  <si>
-    <t>API-010</t>
-  </si>
-  <si>
-    <t>API-011</t>
-  </si>
-  <si>
     <t>API-03, FR-03</t>
   </si>
   <si>
@@ -2194,24 +2131,6 @@
     <t>Verify offender trail points are returned in chronological order</t>
   </si>
   <si>
-    <t>API-012</t>
-  </si>
-  <si>
-    <t>API-013</t>
-  </si>
-  <si>
-    <t>API-014</t>
-  </si>
-  <si>
-    <t>API-015</t>
-  </si>
-  <si>
-    <t>API-016</t>
-  </si>
-  <si>
-    <t>API-017</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">1. Send </t>
     </r>
@@ -2247,6 +2166,758 @@
     <t>An offender with existing trail points is available and a valid new location point can be added.</t>
   </si>
   <si>
+    <t>The newly added point is present in the trail, and the complete trail is still returned in chronological order from oldest to newest.</t>
+  </si>
+  <si>
+    <t>Verify stats endpoint matches current system data</t>
+  </si>
+  <si>
+    <t>Offender and trail data exist in the system.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Send </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>GET /api/stats</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. 2. Retrieve the offender list and relevant trail data through the API. 3. Independently calculate total offenders, Active offenders and total trail points. 4. Compare the calculated values with the stats response.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The values returned by </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>GET /api/stats</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> match the totals independently calculated from the current stored data.</t>
+    </r>
+  </si>
+  <si>
+    <t>API-05, API-02, FR-11</t>
+  </si>
+  <si>
+    <t>Verify stats update after offender creation</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Send </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>GET /api/stats</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and record the current offender and Active offender totals. 2. Create a valid offender using </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>POST /api/offenders</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> with a known status. 3. Send </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>GET /api/stats</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> again. 4. Compare the before and after values.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Total offenders increases by </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. If the new offender is Active, Active offenders also increases by </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; if Inactive, the Active count remains unchanged.</t>
+    </r>
+  </si>
+  <si>
+    <t>API-05, API-02, FR-05, FR-11</t>
+  </si>
+  <si>
+    <t>Verify stats update after deleting an offender with trail data</t>
+  </si>
+  <si>
+    <t>An existing offender with a known status and known number of trail points is available.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Retrieve the offender's trail and record the number of trail points. 2. Send </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>GET /api/stats</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and record the current totals. 3. Delete the offender using </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>DELETE /api/offenders/{id}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. 4. Send </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>GET /api/stats</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> again. 5. Compare the before and after values.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Total offenders decreases by </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. If the deleted offender was Active, Active offenders decreases by </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. Total trail points decreases by exactly the number of trail points that belonged to the deleted offender.</t>
+    </r>
+  </si>
+  <si>
+    <t>API-05, FR-04, FR-11</t>
+  </si>
+  <si>
+    <t>Verify offender counts remain unchanged after updating an offender</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Send </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>GET /api/stats</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and record the current Total Offenders and Active Offenders values. 2. Send </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>PUT /api/offenders/{id}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to modify a field other than Status, such as First Name or Last Name. 3. Verify the update succeeds. 4. Send </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>GET /api/stats</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> again. 5. Compare the before and after values.</t>
+    </r>
+  </si>
+  <si>
+    <t>The offender is updated successfully. Total Offenders remains unchanged. Active Offenders also remains unchanged because the offender's Status was not modified.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Send </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>POST /api/offenders/{id}/locations</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> with an otherwise valid payload and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>speedKmh = -1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. 2. Repeat with </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>batteryPct = -1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. 3. Repeat with </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>batteryPct = 101</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. 4. Repeat with </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>signal = 0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. 5. Repeat with </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>signal = 6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. 6. Repeat with latitude or longitude outside the standard geographic coordinate ranges, for example </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>lat = 91</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> or </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>lon = 181</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. 7. Record the HTTP status code and response body for each request. 8. Retrieve the offender's trail using </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>GET /api/offenders/{id}/trail</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and verify that none of the invalid location points were persisted.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Each invalid request returns HTTP </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>400 Bad Request</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> with an error description, and none of the invalid location points are persisted. For the coordinate cases, the numeric boundaries used are a reasonable testing assumption based on standard geographic coordinate ranges, because FR-10 requires valid coordinates but does not explicitly define their numeric limits.</t>
+    </r>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>BUG-001</t>
+  </si>
+  <si>
+    <t>BUG-002</t>
+  </si>
+  <si>
+    <t>Positive</t>
+  </si>
+  <si>
+    <t>BUG-003</t>
+  </si>
+  <si>
+    <t>BUG-004</t>
+  </si>
+  <si>
+    <t>BUG-005</t>
+  </si>
+  <si>
+    <t>BUG-006</t>
+  </si>
+  <si>
+    <t>BUG-007</t>
+  </si>
+  <si>
+    <t>UI-041</t>
+  </si>
+  <si>
+    <t>UI-042</t>
+  </si>
+  <si>
+    <t>UI-043</t>
+  </si>
+  <si>
+    <t>UI-044</t>
+  </si>
+  <si>
+    <t>UI-045</t>
+  </si>
+  <si>
+    <t>UI-046</t>
+  </si>
+  <si>
+    <t>UI-047</t>
+  </si>
+  <si>
+    <t>UI-048</t>
+  </si>
+  <si>
+    <t>UI-049</t>
+  </si>
+  <si>
+    <t>UI-050</t>
+  </si>
+  <si>
+    <t>UI-051</t>
+  </si>
+  <si>
+    <t>UI-052</t>
+  </si>
+  <si>
+    <t>UI-053</t>
+  </si>
+  <si>
+    <t>UI-054</t>
+  </si>
+  <si>
+    <t>UI-055</t>
+  </si>
+  <si>
+    <t>UI-056</t>
+  </si>
+  <si>
+    <t>UI-057</t>
+  </si>
+  <si>
+    <t>UI-058</t>
+  </si>
+  <si>
+    <t>UI-059</t>
+  </si>
+  <si>
+    <t>UI-060</t>
+  </si>
+  <si>
+    <t>UI-061</t>
+  </si>
+  <si>
+    <t>BUG-008</t>
+  </si>
+  <si>
+    <t>BUG-009</t>
+  </si>
+  <si>
+    <t>Select an existing offender with a Date of Birth.
+Retrieve the offender through the API and record the stored Date of Birth.
+Open the same offender in the UI.
+Compare the displayed Date of Birth with the API value.</t>
+  </si>
+  <si>
+    <t>BUG-010</t>
+  </si>
+  <si>
+    <t>BUG-011</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Blocked</t>
+  </si>
+  <si>
+    <t>Trail point details displayed on the map and in the Trail Points table match the corresponding API records for the tested points. API timestamps are returned in UTC, while the UI displays the equivalent local time (UTC+3). Coordinate values are displayed with reduced decimal precision in the UI but represent the same locations.</t>
+  </si>
+  <si>
+    <t>BUG-012</t>
+  </si>
+  <si>
+    <t>BUG-013</t>
+  </si>
+  <si>
+    <t>1. Open the Add Location form for an existing offender.
+2. Enter valid values for latitude, longitude, battery, and signal.
+3. Enter a negative speed value, for example -1.
+4. Attempt to save the location point.</t>
+  </si>
+  <si>
+    <t>1. Open the Add Location form for an existing offender.
+2. Enter valid values for all location fields.
+3. Replace either the latitude or longitude with a value outside the valid coordinate range.
+4. Attempt to save the location point.</t>
+  </si>
+  <si>
+    <t>BUG-014</t>
+  </si>
+  <si>
+    <t>1. Open the Add Location form for an existing offender. 2. Enter otherwise valid location data with battery below 0 and attempt to save. 3. Repeat with battery above 100.</t>
+  </si>
+  <si>
+    <t>1. Open the Add Location form for an existing offender. 2. Enter otherwise valid location data with signal below 1 and attempt to save. 3. Repeat with signal above 5.</t>
+  </si>
+  <si>
+    <t>BUG-015</t>
+  </si>
+  <si>
+    <t>After deleting an offender with associated trail data, the offender was removed, but the total trail point count did not decrease to reflect the deletion. See BUG-008.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The default pagination metadata is inconsistent. The returned </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>totalPages</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> value does not match </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>ceil(total / pageSize)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. See BUG-001.</t>
+    </r>
+  </si>
+  <si>
+    <t>API reports totalPages=6 for 33 offenders with pageSize=5. Following the reported pagination provides access to only 30 offenders; page 7 can be requested directly and returns the remaining 3.</t>
+  </si>
+  <si>
+    <t>BUG-016</t>
+  </si>
+  <si>
+    <t>BUG-017</t>
+  </si>
+  <si>
+    <t>POST accepted an offender payload with a missing required field and returned HTTP 201 instead of rejecting the request with HTTP 400.</t>
+  </si>
+  <si>
+    <t>POST accepted an offender payload with an existing National ID instead of rejecting the duplicate.</t>
+  </si>
+  <si>
+    <t>POST accepted an offender payload with a future Date of Birth instead of rejecting it.</t>
+  </si>
+  <si>
+    <t>PUT accepted an update containing a duplicate National ID instead of rejecting the invalid update.</t>
+  </si>
+  <si>
+    <t>BUG-013, BUG-014, BUG-015</t>
+  </si>
+  <si>
+    <t>API accepted and persisted multiple invalid location values, including negative speed, negative battery, signal=6, and latitude=91, instead of rejecting them with HTTP 400.</t>
+  </si>
+  <si>
+    <t>Trail points were returned in a non-chronological order instead of oldest to newest.</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">1. Retrieve the offender's current trail using </t>
     </r>
@@ -2256,7 +2927,7 @@
         <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
       </rPr>
-      <t>GET /api/offenders/{id}/trail</t>
+      <t>GET /api/offenders/{id}/location</t>
     </r>
     <r>
       <rPr>
@@ -2274,7 +2945,7 @@
         <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
       </rPr>
-      <t>POST /api/offenders/{id}/trail</t>
+      <t>POST /api/offenders/{id}/location</t>
     </r>
     <r>
       <rPr>
@@ -2288,547 +2959,13 @@
     </r>
   </si>
   <si>
-    <t>The newly added point is present in the trail, and the complete trail is still returned in chronological order from oldest to newest.</t>
-  </si>
-  <si>
-    <t>Verify stats endpoint matches current system data</t>
-  </si>
-  <si>
-    <t>Offender and trail data exist in the system.</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. Send </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>GET /api/stats</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>. 2. Retrieve the offender list and relevant trail data through the API. 3. Independently calculate total offenders, Active offenders and total trail points. 4. Compare the calculated values with the stats response.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">The values returned by </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>GET /api/stats</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> match the totals independently calculated from the current stored data.</t>
-    </r>
-  </si>
-  <si>
-    <t>API-05, API-02, FR-11</t>
-  </si>
-  <si>
-    <t>Verify stats update after offender creation</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. Send </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>GET /api/stats</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> and record the current offender and Active offender totals. 2. Create a valid offender using </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>POST /api/offenders</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> with a known status. 3. Send </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>GET /api/stats</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> again. 4. Compare the before and after values.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Total offenders increases by </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. If the new offender is Active, Active offenders also increases by </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>; if Inactive, the Active count remains unchanged.</t>
-    </r>
-  </si>
-  <si>
-    <t>API-05, API-02, FR-05, FR-11</t>
-  </si>
-  <si>
-    <t>Verify stats update after deleting an offender with trail data</t>
-  </si>
-  <si>
-    <t>An existing offender with a known status and known number of trail points is available.</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. Retrieve the offender's trail and record the number of trail points. 2. Send </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>GET /api/stats</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> and record the current totals. 3. Delete the offender using </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>DELETE /api/offenders/{id}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. 4. Send </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>GET /api/stats</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> again. 5. Compare the before and after values.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Total offenders decreases by </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. If the deleted offender was Active, Active offenders decreases by </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>. Total trail points decreases by exactly the number of trail points that belonged to the deleted offender.</t>
-    </r>
-  </si>
-  <si>
-    <t>API-05, FR-04, FR-11</t>
-  </si>
-  <si>
-    <t>Verify offender counts remain unchanged after updating an offender</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. Send </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>GET /api/stats</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> and record the current Total Offenders and Active Offenders values. 2. Send </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>PUT /api/offenders/{id}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> to modify a field other than Status, such as First Name or Last Name. 3. Verify the update succeeds. 4. Send </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>GET /api/stats</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> again. 5. Compare the before and after values.</t>
-    </r>
-  </si>
-  <si>
-    <t>The offender is updated successfully. Total Offenders remains unchanged. Active Offenders also remains unchanged because the offender's Status was not modified.</t>
-  </si>
-  <si>
-    <t>API-018</t>
-  </si>
-  <si>
-    <t>API-019</t>
-  </si>
-  <si>
-    <t>API-020</t>
-  </si>
-  <si>
-    <t>API-021</t>
-  </si>
-  <si>
-    <t>API-022</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. Send </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>POST /api/offenders/{id}/locations</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> with an otherwise valid payload and </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>speedKmh = -1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. 2. Repeat with </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>batteryPct = -1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. 3. Repeat with </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>batteryPct = 101</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. 4. Repeat with </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>signal = 0</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. 5. Repeat with </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>signal = 6</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. 6. Repeat with latitude or longitude outside the standard geographic coordinate ranges, for example </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>lat = 91</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> or </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>lon = 181</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. 7. Record the HTTP status code and response body for each request. 8. Retrieve the offender's trail using </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>GET /api/offenders/{id}/trail</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> and verify that none of the invalid location points were persisted.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Each invalid request returns HTTP </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial Unicode MS"/>
-      </rPr>
-      <t>400 Bad Request</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> with an error description, and none of the invalid location points are persisted. For the coordinate cases, the numeric boundaries used are a reasonable testing assumption based on standard geographic coordinate ranges, because FR-10 requires valid coordinates but does not explicitly define their numeric limits.</t>
-    </r>
+    <t>Trail ordering is already non-chronological before adding a new location point; the API does not maintain oldest-to-newest ordering. See BUG-011.</t>
+  </si>
+  <si>
+    <t>After deleting an offender with trail data, the offender count decreased but the total trail point count did not decrease because the offender's trail data remained in the system.</t>
+  </si>
+  <si>
+    <t>selecting the current date in the UI changes the DOB to the previous month, preventing validation of the current-date boundary condition. See BUG-010.</t>
   </si>
 </sst>
 </file>
@@ -2875,7 +3012,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2890,7 +3027,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3205,14 +3350,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{353BE5A4-5F86-4F9D-AC72-525DD816882D}">
-  <dimension ref="A1:K63"/>
+  <dimension ref="A1:L62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="15.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="221.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="255.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3238,7 +3384,7 @@
         <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J1" t="s">
         <v>8</v>
@@ -3246,25 +3392,28 @@
       <c r="K1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" ht="45">
+      <c r="L1" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="45">
       <c r="A2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
       </c>
       <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>18</v>
       </c>
       <c r="G2" t="s">
         <v>11</v>
@@ -3273,33 +3422,33 @@
         <v>12</v>
       </c>
       <c r="I2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J2" t="s">
+        <v>305</v>
+      </c>
+      <c r="K2" t="s">
         <v>13</v>
       </c>
-      <c r="K2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="60">
+    </row>
+    <row r="3" spans="1:12" ht="60">
       <c r="A3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B3" t="s">
         <v>10</v>
       </c>
       <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" t="s">
         <v>20</v>
-      </c>
-      <c r="F3" t="s">
-        <v>21</v>
       </c>
       <c r="G3" t="s">
         <v>11</v>
@@ -3308,33 +3457,33 @@
         <v>12</v>
       </c>
       <c r="I3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J3" t="s">
-        <v>13</v>
+        <v>306</v>
       </c>
       <c r="K3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="60">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="60">
       <c r="A4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B4" t="s">
         <v>10</v>
       </c>
       <c r="C4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" t="s">
         <v>22</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" t="s">
         <v>23</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" t="s">
-        <v>24</v>
       </c>
       <c r="G4" t="s">
         <v>11</v>
@@ -3343,33 +3492,33 @@
         <v>12</v>
       </c>
       <c r="I4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J4" t="s">
+        <v>305</v>
+      </c>
+      <c r="K4" t="s">
         <v>13</v>
       </c>
-      <c r="K4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="45">
+    </row>
+    <row r="5" spans="1:12" ht="45">
       <c r="A5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" t="s">
         <v>26</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>27</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="F5" t="s">
         <v>29</v>
-      </c>
-      <c r="F5" t="s">
-        <v>30</v>
       </c>
       <c r="G5" t="s">
         <v>11</v>
@@ -3378,33 +3527,33 @@
         <v>12</v>
       </c>
       <c r="I5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J5" t="s">
+        <v>305</v>
+      </c>
+      <c r="K5" t="s">
         <v>13</v>
       </c>
-      <c r="K5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11">
+    </row>
+    <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" t="s">
         <v>31</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>32</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>33</v>
-      </c>
-      <c r="F6" t="s">
-        <v>34</v>
       </c>
       <c r="G6" t="s">
         <v>11</v>
@@ -3413,33 +3562,33 @@
         <v>12</v>
       </c>
       <c r="I6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J6" t="s">
+        <v>305</v>
+      </c>
+      <c r="K6" t="s">
         <v>13</v>
       </c>
-      <c r="K6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11">
+    </row>
+    <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" t="s">
         <v>35</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>36</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>37</v>
-      </c>
-      <c r="F7" t="s">
-        <v>38</v>
       </c>
       <c r="G7" t="s">
         <v>11</v>
@@ -3448,33 +3597,33 @@
         <v>12</v>
       </c>
       <c r="I7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J7" t="s">
+        <v>305</v>
+      </c>
+      <c r="K7" t="s">
         <v>13</v>
       </c>
-      <c r="K7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11">
+    </row>
+    <row r="8" spans="1:12">
       <c r="A8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" t="s">
         <v>39</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>40</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>41</v>
-      </c>
-      <c r="F8" t="s">
-        <v>42</v>
       </c>
       <c r="G8" t="s">
         <v>11</v>
@@ -3483,68 +3632,68 @@
         <v>12</v>
       </c>
       <c r="I8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J8" t="s">
-        <v>13</v>
+        <v>306</v>
       </c>
       <c r="K8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
       <c r="A9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C9" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" t="s">
         <v>43</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>44</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>45</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>46</v>
-      </c>
-      <c r="G9" t="s">
-        <v>47</v>
       </c>
       <c r="H9" t="s">
         <v>12</v>
       </c>
       <c r="I9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J9" t="s">
+        <v>305</v>
+      </c>
+      <c r="K9" t="s">
         <v>13</v>
       </c>
-      <c r="K9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11">
+    </row>
+    <row r="10" spans="1:12">
       <c r="A10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B10" t="s">
+        <v>50</v>
+      </c>
+      <c r="C10" t="s">
         <v>51</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>52</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>53</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>54</v>
-      </c>
-      <c r="F10" t="s">
-        <v>55</v>
       </c>
       <c r="G10" t="s">
         <v>11</v>
@@ -3553,33 +3702,33 @@
         <v>12</v>
       </c>
       <c r="I10" t="s">
-        <v>48</v>
+        <v>309</v>
       </c>
       <c r="J10" t="s">
+        <v>305</v>
+      </c>
+      <c r="K10" t="s">
         <v>13</v>
       </c>
-      <c r="K10" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11">
+    </row>
+    <row r="11" spans="1:12">
       <c r="A11" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C11" t="s">
+        <v>55</v>
+      </c>
+      <c r="D11" t="s">
         <v>56</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>57</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>58</v>
-      </c>
-      <c r="F11" t="s">
-        <v>59</v>
       </c>
       <c r="G11" t="s">
         <v>11</v>
@@ -3588,33 +3737,33 @@
         <v>12</v>
       </c>
       <c r="I11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J11" t="s">
-        <v>13</v>
+        <v>306</v>
       </c>
       <c r="K11" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
       <c r="A12" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C12" t="s">
+        <v>59</v>
+      </c>
+      <c r="D12" t="s">
         <v>60</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>61</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>62</v>
-      </c>
-      <c r="F12" t="s">
-        <v>63</v>
       </c>
       <c r="G12" t="s">
         <v>11</v>
@@ -3623,33 +3772,33 @@
         <v>12</v>
       </c>
       <c r="I12" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J12" t="s">
-        <v>13</v>
+        <v>306</v>
       </c>
       <c r="K12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
       <c r="A13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" t="s">
+        <v>56</v>
+      </c>
+      <c r="E13" t="s">
         <v>64</v>
       </c>
-      <c r="D13" t="s">
-        <v>57</v>
-      </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>65</v>
-      </c>
-      <c r="F13" t="s">
-        <v>66</v>
       </c>
       <c r="G13" t="s">
         <v>11</v>
@@ -3658,103 +3807,106 @@
         <v>12</v>
       </c>
       <c r="I13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J13" t="s">
-        <v>13</v>
+        <v>306</v>
       </c>
       <c r="K13" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
       <c r="A14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C14" t="s">
+        <v>66</v>
+      </c>
+      <c r="D14" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" t="s">
         <v>67</v>
       </c>
-      <c r="D14" t="s">
-        <v>57</v>
-      </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>68</v>
       </c>
-      <c r="F14" t="s">
-        <v>69</v>
-      </c>
       <c r="G14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H14" t="s">
         <v>12</v>
       </c>
       <c r="I14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J14" t="s">
+        <v>305</v>
+      </c>
+      <c r="K14" t="s">
         <v>13</v>
       </c>
-      <c r="K14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11">
+    </row>
+    <row r="15" spans="1:12">
       <c r="A15" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B15" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C15" t="s">
+        <v>82</v>
+      </c>
+      <c r="D15" t="s">
+        <v>56</v>
+      </c>
+      <c r="E15" t="s">
         <v>83</v>
       </c>
-      <c r="D15" t="s">
-        <v>57</v>
-      </c>
-      <c r="E15" t="s">
+      <c r="F15" t="s">
         <v>84</v>
       </c>
-      <c r="F15" t="s">
-        <v>85</v>
-      </c>
       <c r="G15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H15" t="s">
         <v>12</v>
       </c>
       <c r="I15" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J15" t="s">
+        <v>342</v>
+      </c>
+      <c r="K15" t="s">
         <v>13</v>
       </c>
-      <c r="K15" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11">
+      <c r="L15" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12">
       <c r="A16" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B16" t="s">
+        <v>87</v>
+      </c>
+      <c r="C16" t="s">
         <v>88</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>89</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>90</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>91</v>
-      </c>
-      <c r="F16" t="s">
-        <v>92</v>
       </c>
       <c r="G16" t="s">
         <v>11</v>
@@ -3763,33 +3915,33 @@
         <v>12</v>
       </c>
       <c r="I16" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J16" t="s">
+        <v>305</v>
+      </c>
+      <c r="K16" t="s">
         <v>13</v>
       </c>
-      <c r="K16" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11">
+    </row>
+    <row r="17" spans="1:12">
       <c r="A17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B17" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C17" t="s">
+        <v>92</v>
+      </c>
+      <c r="D17" t="s">
         <v>93</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>94</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>95</v>
-      </c>
-      <c r="F17" t="s">
-        <v>96</v>
       </c>
       <c r="G17" t="s">
         <v>11</v>
@@ -3798,33 +3950,33 @@
         <v>12</v>
       </c>
       <c r="I17" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J17" t="s">
-        <v>13</v>
+        <v>306</v>
       </c>
       <c r="K17" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12">
       <c r="A18" t="s">
+        <v>98</v>
+      </c>
+      <c r="B18" t="s">
+        <v>103</v>
+      </c>
+      <c r="C18" t="s">
         <v>99</v>
       </c>
-      <c r="B18" t="s">
-        <v>104</v>
-      </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>100</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>101</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>102</v>
-      </c>
-      <c r="F18" t="s">
-        <v>103</v>
       </c>
       <c r="G18" t="s">
         <v>11</v>
@@ -3833,33 +3985,33 @@
         <v>12</v>
       </c>
       <c r="I18" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J18" t="s">
-        <v>13</v>
+        <v>306</v>
       </c>
       <c r="K18" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12">
       <c r="A19" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B19" t="s">
+        <v>120</v>
+      </c>
+      <c r="C19" t="s">
         <v>104</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>105</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>106</v>
       </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
         <v>107</v>
-      </c>
-      <c r="F19" t="s">
-        <v>108</v>
       </c>
       <c r="G19" t="s">
         <v>11</v>
@@ -3868,33 +4020,33 @@
         <v>12</v>
       </c>
       <c r="I19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J19" t="s">
+        <v>305</v>
+      </c>
+      <c r="K19" t="s">
         <v>13</v>
       </c>
-      <c r="K19" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11">
+    </row>
+    <row r="20" spans="1:12">
       <c r="A20" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B20" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C20" t="s">
+        <v>108</v>
+      </c>
+      <c r="D20" t="s">
+        <v>105</v>
+      </c>
+      <c r="E20" t="s">
         <v>109</v>
       </c>
-      <c r="D20" t="s">
+      <c r="F20" t="s">
         <v>110</v>
-      </c>
-      <c r="E20" t="s">
-        <v>111</v>
-      </c>
-      <c r="F20" t="s">
-        <v>112</v>
       </c>
       <c r="G20" t="s">
         <v>11</v>
@@ -3903,126 +4055,126 @@
         <v>12</v>
       </c>
       <c r="I20" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="J20" t="s">
+        <v>305</v>
+      </c>
+      <c r="K20" t="s">
         <v>13</v>
       </c>
-      <c r="K20" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11">
+    </row>
+    <row r="21" spans="1:12">
       <c r="A21" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="B21" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C21" t="s">
+        <v>111</v>
+      </c>
+      <c r="D21" t="s">
+        <v>112</v>
+      </c>
+      <c r="E21" t="s">
         <v>113</v>
       </c>
-      <c r="D21" t="s">
-        <v>110</v>
-      </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>114</v>
-      </c>
-      <c r="F21" t="s">
-        <v>115</v>
       </c>
       <c r="G21" t="s">
         <v>11</v>
       </c>
       <c r="H21" t="s">
+        <v>115</v>
+      </c>
+      <c r="I21" t="s">
+        <v>47</v>
+      </c>
+      <c r="J21" t="s">
+        <v>306</v>
+      </c>
+      <c r="K21" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12">
+      <c r="A22" t="s">
+        <v>119</v>
+      </c>
+      <c r="B22" t="s">
+        <v>121</v>
+      </c>
+      <c r="C22" t="s">
+        <v>122</v>
+      </c>
+      <c r="D22" t="s">
+        <v>123</v>
+      </c>
+      <c r="E22" t="s">
+        <v>124</v>
+      </c>
+      <c r="F22" t="s">
+        <v>125</v>
+      </c>
+      <c r="G22" t="s">
+        <v>46</v>
+      </c>
+      <c r="H22" t="s">
         <v>12</v>
       </c>
-      <c r="I21" t="s">
-        <v>48</v>
-      </c>
-      <c r="J21" t="s">
-        <v>13</v>
-      </c>
-      <c r="K21" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11">
-      <c r="A22" t="s">
-        <v>124</v>
-      </c>
-      <c r="B22" t="s">
-        <v>125</v>
-      </c>
-      <c r="C22" t="s">
-        <v>116</v>
-      </c>
-      <c r="D22" t="s">
-        <v>117</v>
-      </c>
-      <c r="E22" t="s">
-        <v>118</v>
-      </c>
-      <c r="F22" t="s">
-        <v>119</v>
-      </c>
-      <c r="G22" t="s">
+      <c r="I22" t="s">
+        <v>47</v>
+      </c>
+      <c r="J22" t="s">
+        <v>306</v>
+      </c>
+      <c r="K22" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" ht="60">
+      <c r="A23" t="s">
+        <v>129</v>
+      </c>
+      <c r="B23" t="s">
+        <v>121</v>
+      </c>
+      <c r="C23" t="s">
+        <v>126</v>
+      </c>
+      <c r="D23" t="s">
+        <v>127</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="F23" t="s">
+        <v>128</v>
+      </c>
+      <c r="G23" t="s">
         <v>11</v>
       </c>
-      <c r="H22" t="s">
-        <v>120</v>
-      </c>
-      <c r="I22" t="s">
-        <v>48</v>
-      </c>
-      <c r="J22" t="s">
-        <v>13</v>
-      </c>
-      <c r="K22" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11">
-      <c r="A23" t="s">
-        <v>135</v>
-      </c>
-      <c r="B23" t="s">
-        <v>126</v>
-      </c>
-      <c r="C23" t="s">
-        <v>127</v>
-      </c>
-      <c r="D23" t="s">
-        <v>128</v>
-      </c>
-      <c r="E23" t="s">
-        <v>129</v>
-      </c>
-      <c r="F23" t="s">
+      <c r="H23" t="s">
+        <v>115</v>
+      </c>
+      <c r="I23" t="s">
+        <v>47</v>
+      </c>
+      <c r="J23" t="s">
+        <v>306</v>
+      </c>
+      <c r="K23" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12">
+      <c r="A24" t="s">
         <v>130</v>
       </c>
-      <c r="G23" t="s">
-        <v>47</v>
-      </c>
-      <c r="H23" t="s">
-        <v>12</v>
-      </c>
-      <c r="I23" t="s">
-        <v>48</v>
-      </c>
-      <c r="J23" t="s">
-        <v>13</v>
-      </c>
-      <c r="K23" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11">
-      <c r="A24" t="s">
-        <v>136</v>
-      </c>
       <c r="B24" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="C24" t="s">
         <v>131</v>
@@ -4030,101 +4182,107 @@
       <c r="D24" t="s">
         <v>132</v>
       </c>
-      <c r="E24" s="3" t="s">
-        <v>134</v>
+      <c r="E24" t="s">
+        <v>145</v>
       </c>
       <c r="F24" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="G24" t="s">
         <v>11</v>
       </c>
       <c r="H24" t="s">
-        <v>120</v>
+        <v>12</v>
       </c>
       <c r="I24" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J24" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12">
       <c r="A25" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="B25" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="C25" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="D25" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="E25" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="F25" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
       <c r="G25" t="s">
         <v>11</v>
       </c>
       <c r="H25" t="s">
-        <v>12</v>
+        <v>115</v>
       </c>
       <c r="I25" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J25" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11">
+        <v>306</v>
+      </c>
+      <c r="K25" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12">
       <c r="A26" t="s">
+        <v>138</v>
+      </c>
+      <c r="B26" t="s">
+        <v>140</v>
+      </c>
+      <c r="C26" t="s">
+        <v>135</v>
+      </c>
+      <c r="D26" t="s">
+        <v>136</v>
+      </c>
+      <c r="E26" t="s">
+        <v>143</v>
+      </c>
+      <c r="F26" t="s">
         <v>144</v>
-      </c>
-      <c r="B26" t="s">
-        <v>146</v>
-      </c>
-      <c r="C26" t="s">
-        <v>139</v>
-      </c>
-      <c r="D26" t="s">
-        <v>140</v>
-      </c>
-      <c r="E26" t="s">
-        <v>147</v>
-      </c>
-      <c r="F26" t="s">
-        <v>148</v>
       </c>
       <c r="G26" t="s">
         <v>11</v>
       </c>
       <c r="H26" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I26" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J26" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11">
+        <v>306</v>
+      </c>
+      <c r="K26" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12">
       <c r="A27" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="B27" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C27" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="D27" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="E27" t="s">
         <v>149</v>
@@ -4136,27 +4294,27 @@
         <v>11</v>
       </c>
       <c r="H27" t="s">
-        <v>120</v>
+        <v>12</v>
       </c>
       <c r="I27" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J27" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12">
       <c r="A28" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="B28" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="C28" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D28" t="s">
-        <v>154</v>
+        <v>134</v>
       </c>
       <c r="E28" t="s">
         <v>155</v>
@@ -4168,94 +4326,100 @@
         <v>11</v>
       </c>
       <c r="H28" t="s">
-        <v>12</v>
+        <v>115</v>
       </c>
       <c r="I28" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J28" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11">
+        <v>305</v>
+      </c>
+      <c r="L28" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12">
       <c r="A29" t="s">
+        <v>152</v>
+      </c>
+      <c r="B29" t="s">
+        <v>160</v>
+      </c>
+      <c r="C29" t="s">
+        <v>157</v>
+      </c>
+      <c r="E29" t="s">
         <v>158</v>
       </c>
-      <c r="B29" t="s">
+      <c r="F29" s="5" t="s">
         <v>159</v>
-      </c>
-      <c r="C29" t="s">
-        <v>160</v>
-      </c>
-      <c r="D29" t="s">
-        <v>140</v>
-      </c>
-      <c r="E29" t="s">
-        <v>161</v>
-      </c>
-      <c r="F29" t="s">
-        <v>162</v>
       </c>
       <c r="G29" t="s">
         <v>11</v>
       </c>
       <c r="H29" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I29" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J29" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11">
+        <v>306</v>
+      </c>
+      <c r="K29" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12">
       <c r="A30" t="s">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="B30" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="C30" t="s">
+        <v>162</v>
+      </c>
+      <c r="D30" t="s">
         <v>163</v>
       </c>
       <c r="E30" t="s">
         <v>164</v>
       </c>
-      <c r="F30" s="5" t="s">
+      <c r="F30" t="s">
         <v>165</v>
       </c>
       <c r="G30" t="s">
         <v>11</v>
       </c>
       <c r="H30" t="s">
-        <v>120</v>
+        <v>12</v>
       </c>
       <c r="I30" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J30" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" ht="60">
       <c r="A31" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="B31" t="s">
+        <v>161</v>
+      </c>
+      <c r="C31" t="s">
+        <v>166</v>
+      </c>
+      <c r="D31" t="s">
         <v>167</v>
       </c>
-      <c r="C31" t="s">
+      <c r="E31" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="F31" t="s">
         <v>168</v>
-      </c>
-      <c r="D31" t="s">
-        <v>169</v>
-      </c>
-      <c r="E31" t="s">
-        <v>170</v>
-      </c>
-      <c r="F31" t="s">
-        <v>171</v>
       </c>
       <c r="G31" t="s">
         <v>11</v>
@@ -4264,30 +4428,33 @@
         <v>12</v>
       </c>
       <c r="I31" t="s">
-        <v>48</v>
+        <v>169</v>
       </c>
       <c r="J31" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11">
+        <v>306</v>
+      </c>
+      <c r="K31" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" ht="60">
       <c r="A32" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="B32" t="s">
+        <v>161</v>
+      </c>
+      <c r="C32" t="s">
+        <v>170</v>
+      </c>
+      <c r="D32" t="s">
         <v>167</v>
       </c>
-      <c r="C32" t="s">
-        <v>172</v>
-      </c>
-      <c r="D32" t="s">
-        <v>173</v>
-      </c>
-      <c r="E32" t="s">
-        <v>174</v>
+      <c r="E32" s="3" t="s">
+        <v>346</v>
       </c>
       <c r="F32" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="G32" t="s">
         <v>11</v>
@@ -4296,30 +4463,33 @@
         <v>12</v>
       </c>
       <c r="I32" t="s">
-        <v>176</v>
+        <v>85</v>
       </c>
       <c r="J32" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9">
+        <v>306</v>
+      </c>
+      <c r="K32" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12">
       <c r="A33" t="s">
-        <v>192</v>
+        <v>182</v>
       </c>
       <c r="B33" t="s">
+        <v>161</v>
+      </c>
+      <c r="C33" t="s">
+        <v>172</v>
+      </c>
+      <c r="D33" t="s">
         <v>167</v>
       </c>
-      <c r="C33" t="s">
-        <v>177</v>
-      </c>
-      <c r="D33" t="s">
+      <c r="E33" t="s">
+        <v>349</v>
+      </c>
+      <c r="F33" t="s">
         <v>173</v>
-      </c>
-      <c r="E33" t="s">
-        <v>178</v>
-      </c>
-      <c r="F33" t="s">
-        <v>179</v>
       </c>
       <c r="G33" t="s">
         <v>11</v>
@@ -4328,27 +4498,33 @@
         <v>12</v>
       </c>
       <c r="I33" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9">
+        <v>85</v>
+      </c>
+      <c r="J33" t="s">
+        <v>306</v>
+      </c>
+      <c r="K33" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12">
       <c r="A34" t="s">
-        <v>193</v>
+        <v>183</v>
       </c>
       <c r="B34" t="s">
+        <v>161</v>
+      </c>
+      <c r="C34" t="s">
+        <v>174</v>
+      </c>
+      <c r="D34" t="s">
         <v>167</v>
       </c>
-      <c r="C34" t="s">
-        <v>180</v>
-      </c>
-      <c r="D34" t="s">
+      <c r="E34" t="s">
+        <v>350</v>
+      </c>
+      <c r="F34" t="s">
         <v>173</v>
-      </c>
-      <c r="E34" t="s">
-        <v>181</v>
-      </c>
-      <c r="F34" t="s">
-        <v>182</v>
       </c>
       <c r="G34" t="s">
         <v>11</v>
@@ -4357,160 +4533,187 @@
         <v>12</v>
       </c>
       <c r="I34" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9">
+        <v>85</v>
+      </c>
+      <c r="K34" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12">
       <c r="A35" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="B35" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="C35" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="D35" t="s">
-        <v>173</v>
+        <v>132</v>
       </c>
       <c r="E35" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="F35" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="G35" t="s">
         <v>11</v>
       </c>
       <c r="H35" t="s">
-        <v>12</v>
+        <v>115</v>
       </c>
       <c r="I35" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9">
+        <v>178</v>
+      </c>
+      <c r="J35" t="s">
+        <v>306</v>
+      </c>
+      <c r="K35" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12">
       <c r="A36" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="B36" t="s">
-        <v>167</v>
+        <v>186</v>
       </c>
       <c r="C36" t="s">
-        <v>185</v>
-      </c>
-      <c r="D36" s="6" t="s">
-        <v>138</v>
+        <v>187</v>
+      </c>
+      <c r="D36" t="s">
+        <v>188</v>
       </c>
       <c r="E36" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="F36" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="G36" t="s">
         <v>11</v>
       </c>
       <c r="H36" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I36" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9">
+        <v>47</v>
+      </c>
+      <c r="J36" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12">
       <c r="A37" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="B37" t="s">
-        <v>196</v>
+        <v>207</v>
       </c>
       <c r="C37" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="D37" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="E37" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="F37" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="G37" t="s">
         <v>11</v>
       </c>
       <c r="H37" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I37" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9">
+        <v>178</v>
+      </c>
+      <c r="J37" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12">
       <c r="A38" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="B38" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="C38" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="D38" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="E38" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="F38" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="G38" t="s">
         <v>11</v>
       </c>
       <c r="H38" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I38" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9">
+        <v>178</v>
+      </c>
+      <c r="J38" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12">
       <c r="A39" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="B39" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="C39" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="D39" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="E39" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="F39" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="G39" t="s">
         <v>11</v>
       </c>
       <c r="H39" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I39" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9">
+        <v>178</v>
+      </c>
+      <c r="J39" t="s">
+        <v>306</v>
+      </c>
+      <c r="K39" t="s">
+        <v>336</v>
+      </c>
+      <c r="L39" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12">
       <c r="A40" t="s">
-        <v>216</v>
+        <v>206</v>
       </c>
       <c r="B40" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="C40" t="s">
         <v>209</v>
@@ -4528,681 +4731,788 @@
         <v>11</v>
       </c>
       <c r="H40" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="I40" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9">
+        <v>178</v>
+      </c>
+      <c r="J40" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12">
       <c r="A41" t="s">
-        <v>224</v>
+        <v>214</v>
       </c>
       <c r="B41" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="C41" t="s">
+        <v>216</v>
+      </c>
+      <c r="D41" t="s">
+        <v>217</v>
+      </c>
+      <c r="E41" t="s">
+        <v>218</v>
+      </c>
+      <c r="F41" t="s">
         <v>219</v>
-      </c>
-      <c r="D41" t="s">
-        <v>220</v>
-      </c>
-      <c r="E41" t="s">
-        <v>221</v>
-      </c>
-      <c r="F41" t="s">
-        <v>222</v>
       </c>
       <c r="G41" t="s">
         <v>11</v>
       </c>
       <c r="H41" t="s">
-        <v>120</v>
+        <v>220</v>
       </c>
       <c r="I41" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9">
+        <v>47</v>
+      </c>
+      <c r="J41" t="s">
+        <v>306</v>
+      </c>
+      <c r="K41" t="s">
+        <v>307</v>
+      </c>
+      <c r="L41" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12">
       <c r="A42" t="s">
+        <v>315</v>
+      </c>
+      <c r="B42" t="s">
+        <v>215</v>
+      </c>
+      <c r="C42" t="s">
+        <v>222</v>
+      </c>
+      <c r="D42" t="s">
+        <v>223</v>
+      </c>
+      <c r="E42" t="s">
+        <v>224</v>
+      </c>
+      <c r="F42" t="s">
         <v>225</v>
-      </c>
-      <c r="B42" t="s">
-        <v>226</v>
-      </c>
-      <c r="C42" t="s">
-        <v>227</v>
-      </c>
-      <c r="D42" t="s">
-        <v>228</v>
-      </c>
-      <c r="E42" t="s">
-        <v>229</v>
-      </c>
-      <c r="F42" t="s">
-        <v>230</v>
       </c>
       <c r="G42" t="s">
         <v>11</v>
       </c>
       <c r="H42" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="I42" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9">
+        <v>47</v>
+      </c>
+      <c r="J42" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12">
       <c r="A43" t="s">
-        <v>272</v>
+        <v>316</v>
       </c>
       <c r="B43" t="s">
+        <v>215</v>
+      </c>
+      <c r="C43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D43" t="s">
         <v>226</v>
       </c>
-      <c r="C43" t="s">
-        <v>233</v>
-      </c>
-      <c r="D43" t="s">
-        <v>234</v>
-      </c>
       <c r="E43" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="F43" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="G43" t="s">
         <v>11</v>
       </c>
       <c r="H43" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="I43" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9">
+        <v>47</v>
+      </c>
+      <c r="J43" t="s">
+        <v>306</v>
+      </c>
+      <c r="K43" t="s">
+        <v>307</v>
+      </c>
+      <c r="L43" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12">
       <c r="A44" t="s">
-        <v>273</v>
+        <v>317</v>
       </c>
       <c r="B44" t="s">
-        <v>226</v>
+        <v>215</v>
       </c>
       <c r="C44" t="s">
-        <v>19</v>
+        <v>235</v>
       </c>
       <c r="D44" t="s">
+        <v>236</v>
+      </c>
+      <c r="E44" t="s">
         <v>237</v>
       </c>
-      <c r="E44" t="s">
+      <c r="F44" t="s">
         <v>238</v>
-      </c>
-      <c r="F44" t="s">
-        <v>239</v>
       </c>
       <c r="G44" t="s">
         <v>11</v>
       </c>
       <c r="H44" t="s">
+        <v>220</v>
+      </c>
+      <c r="I44" t="s">
+        <v>47</v>
+      </c>
+      <c r="J44" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12">
+      <c r="A45" t="s">
+        <v>318</v>
+      </c>
+      <c r="B45" t="s">
+        <v>215</v>
+      </c>
+      <c r="C45" t="s">
+        <v>229</v>
+      </c>
+      <c r="D45" t="s">
+        <v>230</v>
+      </c>
+      <c r="E45" t="s">
         <v>231</v>
       </c>
-      <c r="I44" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9">
-      <c r="A45" t="s">
-        <v>274</v>
-      </c>
-      <c r="B45" t="s">
-        <v>226</v>
-      </c>
-      <c r="C45" t="s">
-        <v>246</v>
-      </c>
-      <c r="D45" t="s">
-        <v>247</v>
-      </c>
-      <c r="E45" t="s">
-        <v>248</v>
-      </c>
-      <c r="F45" t="s">
-        <v>249</v>
+      <c r="F45" s="1" t="s">
+        <v>232</v>
       </c>
       <c r="G45" t="s">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="H45" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="I45" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="46" spans="1:9">
+      <c r="J45" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12">
       <c r="A46" t="s">
-        <v>275</v>
+        <v>319</v>
       </c>
       <c r="B46" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="C46" t="s">
+        <v>239</v>
+      </c>
+      <c r="D46" t="s">
         <v>240</v>
       </c>
-      <c r="D46" t="s">
+      <c r="E46" t="s">
         <v>241</v>
       </c>
-      <c r="E46" t="s">
+      <c r="F46" t="s">
         <v>242</v>
       </c>
-      <c r="F46" s="1" t="s">
+      <c r="G46" t="s">
+        <v>11</v>
+      </c>
+      <c r="H46" t="s">
+        <v>220</v>
+      </c>
+      <c r="I46" t="s">
+        <v>47</v>
+      </c>
+      <c r="J46" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12">
+      <c r="A47" t="s">
+        <v>320</v>
+      </c>
+      <c r="B47" t="s">
+        <v>221</v>
+      </c>
+      <c r="C47" t="s">
         <v>243</v>
       </c>
-      <c r="G46" t="s">
-        <v>47</v>
-      </c>
-      <c r="H46" t="s">
-        <v>231</v>
-      </c>
-      <c r="I46" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9">
-      <c r="A47" t="s">
-        <v>271</v>
-      </c>
-      <c r="B47" t="s">
-        <v>232</v>
-      </c>
-      <c r="C47" t="s">
-        <v>250</v>
-      </c>
       <c r="D47" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="E47" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="F47" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="G47" t="s">
         <v>11</v>
       </c>
       <c r="H47" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="I47" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9">
+        <v>47</v>
+      </c>
+      <c r="J47" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12">
       <c r="A48" t="s">
-        <v>276</v>
+        <v>321</v>
       </c>
       <c r="B48" t="s">
-        <v>232</v>
+        <v>221</v>
       </c>
       <c r="C48" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="D48" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="E48" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="F48" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="G48" t="s">
         <v>11</v>
       </c>
       <c r="H48" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="I48" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="49" spans="1:9">
+      <c r="J48" t="s">
+        <v>306</v>
+      </c>
+      <c r="K48" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12">
       <c r="A49" t="s">
-        <v>277</v>
+        <v>322</v>
       </c>
       <c r="B49" t="s">
-        <v>232</v>
+        <v>221</v>
       </c>
       <c r="C49" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="D49" t="s">
-        <v>259</v>
+        <v>248</v>
       </c>
       <c r="E49" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
       <c r="F49" t="s">
-        <v>261</v>
+        <v>250</v>
       </c>
       <c r="G49" t="s">
         <v>11</v>
       </c>
       <c r="H49" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="I49" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9">
+        <v>48</v>
+      </c>
+      <c r="J49" t="s">
+        <v>306</v>
+      </c>
+      <c r="K49" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12">
       <c r="A50" t="s">
-        <v>278</v>
+        <v>323</v>
       </c>
       <c r="B50" t="s">
-        <v>232</v>
+        <v>221</v>
       </c>
       <c r="C50" t="s">
-        <v>262</v>
+        <v>253</v>
       </c>
       <c r="D50" t="s">
+        <v>248</v>
+      </c>
+      <c r="E50" t="s">
+        <v>254</v>
+      </c>
+      <c r="F50" t="s">
+        <v>255</v>
+      </c>
+      <c r="G50" t="s">
+        <v>46</v>
+      </c>
+      <c r="H50" t="s">
+        <v>220</v>
+      </c>
+      <c r="I50" t="s">
+        <v>48</v>
+      </c>
+      <c r="J50" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12">
+      <c r="A51" t="s">
+        <v>324</v>
+      </c>
+      <c r="B51" t="s">
+        <v>221</v>
+      </c>
+      <c r="C51" t="s">
+        <v>256</v>
+      </c>
+      <c r="D51" t="s">
+        <v>257</v>
+      </c>
+      <c r="E51" t="s">
+        <v>258</v>
+      </c>
+      <c r="F51" t="s">
         <v>259</v>
       </c>
-      <c r="E50" t="s">
+      <c r="G51" t="s">
+        <v>11</v>
+      </c>
+      <c r="H51" t="s">
+        <v>220</v>
+      </c>
+      <c r="I51" t="s">
+        <v>48</v>
+      </c>
+      <c r="J51" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12">
+      <c r="A52" t="s">
+        <v>325</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="C52" t="s">
         <v>263</v>
       </c>
-      <c r="F50" t="s">
-        <v>261</v>
-      </c>
-      <c r="G50" t="s">
-        <v>11</v>
-      </c>
-      <c r="H50" t="s">
-        <v>231</v>
-      </c>
-      <c r="I50" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9">
-      <c r="A51" t="s">
-        <v>279</v>
-      </c>
-      <c r="B51" t="s">
-        <v>232</v>
-      </c>
-      <c r="C51" t="s">
+      <c r="D52" t="s">
         <v>264</v>
       </c>
-      <c r="D51" t="s">
-        <v>259</v>
-      </c>
-      <c r="E51" t="s">
+      <c r="E52" t="s">
         <v>265</v>
       </c>
-      <c r="F51" t="s">
+      <c r="F52" t="s">
         <v>266</v>
-      </c>
-      <c r="G51" t="s">
-        <v>47</v>
-      </c>
-      <c r="H51" t="s">
-        <v>231</v>
-      </c>
-      <c r="I51" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9">
-      <c r="A52" t="s">
-        <v>280</v>
-      </c>
-      <c r="B52" t="s">
-        <v>232</v>
-      </c>
-      <c r="C52" t="s">
-        <v>267</v>
-      </c>
-      <c r="D52" t="s">
-        <v>268</v>
-      </c>
-      <c r="E52" t="s">
-        <v>269</v>
-      </c>
-      <c r="F52" t="s">
-        <v>270</v>
       </c>
       <c r="G52" t="s">
         <v>11</v>
       </c>
       <c r="H52" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="I52" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9">
+        <v>48</v>
+      </c>
+      <c r="J52" t="s">
+        <v>306</v>
+      </c>
+      <c r="K52" t="s">
+        <v>310</v>
+      </c>
+      <c r="L52" s="7" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12">
       <c r="A53" t="s">
-        <v>301</v>
+        <v>326</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>281</v>
+        <v>260</v>
       </c>
       <c r="C53" t="s">
-        <v>284</v>
+        <v>267</v>
       </c>
       <c r="D53" t="s">
-        <v>285</v>
+        <v>60</v>
       </c>
       <c r="E53" t="s">
-        <v>286</v>
+        <v>268</v>
       </c>
       <c r="F53" t="s">
-        <v>287</v>
+        <v>269</v>
       </c>
       <c r="G53" t="s">
         <v>11</v>
       </c>
       <c r="H53" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="I53" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9">
+        <v>48</v>
+      </c>
+      <c r="J53" t="s">
+        <v>306</v>
+      </c>
+      <c r="K53" t="s">
+        <v>311</v>
+      </c>
+      <c r="L53" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12">
       <c r="A54" t="s">
-        <v>302</v>
+        <v>327</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>281</v>
+        <v>260</v>
       </c>
       <c r="C54" t="s">
-        <v>288</v>
+        <v>270</v>
       </c>
       <c r="D54" t="s">
-        <v>61</v>
+        <v>264</v>
       </c>
       <c r="E54" t="s">
-        <v>289</v>
+        <v>271</v>
       </c>
       <c r="F54" t="s">
-        <v>290</v>
+        <v>266</v>
       </c>
       <c r="G54" t="s">
         <v>11</v>
       </c>
       <c r="H54" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="I54" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9">
+        <v>169</v>
+      </c>
+      <c r="J54" t="s">
+        <v>306</v>
+      </c>
+      <c r="K54" t="s">
+        <v>312</v>
+      </c>
+      <c r="L54" s="6" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12">
       <c r="A55" t="s">
-        <v>303</v>
-      </c>
-      <c r="B55" s="4" t="s">
-        <v>281</v>
+        <v>328</v>
+      </c>
+      <c r="B55" t="s">
+        <v>261</v>
       </c>
       <c r="C55" t="s">
-        <v>291</v>
+        <v>272</v>
       </c>
       <c r="D55" t="s">
-        <v>285</v>
+        <v>273</v>
       </c>
       <c r="E55" t="s">
-        <v>292</v>
+        <v>274</v>
       </c>
       <c r="F55" t="s">
-        <v>287</v>
+        <v>275</v>
       </c>
       <c r="G55" t="s">
         <v>11</v>
       </c>
       <c r="H55" t="s">
-        <v>231</v>
+        <v>276</v>
       </c>
       <c r="I55" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9">
+        <v>48</v>
+      </c>
+      <c r="J55" t="s">
+        <v>306</v>
+      </c>
+      <c r="K55" t="s">
+        <v>314</v>
+      </c>
+      <c r="L55" s="8" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12">
       <c r="A56" t="s">
+        <v>329</v>
+      </c>
+      <c r="B56" t="s">
+        <v>262</v>
+      </c>
+      <c r="C56" t="s">
+        <v>277</v>
+      </c>
+      <c r="D56" t="s">
+        <v>278</v>
+      </c>
+      <c r="E56" t="s">
+        <v>303</v>
+      </c>
+      <c r="F56" t="s">
         <v>304</v>
-      </c>
-      <c r="B56" t="s">
-        <v>282</v>
-      </c>
-      <c r="C56" t="s">
-        <v>293</v>
-      </c>
-      <c r="D56" t="s">
-        <v>294</v>
-      </c>
-      <c r="E56" t="s">
-        <v>295</v>
-      </c>
-      <c r="F56" t="s">
-        <v>296</v>
       </c>
       <c r="G56" t="s">
         <v>11</v>
       </c>
       <c r="H56" t="s">
-        <v>297</v>
+        <v>220</v>
       </c>
       <c r="I56" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9">
+        <v>169</v>
+      </c>
+      <c r="J56" t="s">
+        <v>306</v>
+      </c>
+      <c r="K56" t="s">
+        <v>361</v>
+      </c>
+      <c r="L56" s="7" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12">
       <c r="A57" t="s">
-        <v>305</v>
+        <v>330</v>
       </c>
       <c r="B57" t="s">
-        <v>283</v>
+        <v>233</v>
       </c>
       <c r="C57" t="s">
-        <v>298</v>
+        <v>279</v>
       </c>
       <c r="D57" t="s">
-        <v>299</v>
+        <v>134</v>
       </c>
       <c r="E57" t="s">
-        <v>336</v>
+        <v>280</v>
       </c>
       <c r="F57" t="s">
-        <v>337</v>
+        <v>281</v>
       </c>
       <c r="G57" t="s">
         <v>11</v>
       </c>
       <c r="H57" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="I57" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9">
+        <v>47</v>
+      </c>
+      <c r="J57" t="s">
+        <v>306</v>
+      </c>
+      <c r="K57" t="s">
+        <v>340</v>
+      </c>
+      <c r="L57" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12">
       <c r="A58" t="s">
-        <v>306</v>
+        <v>331</v>
       </c>
       <c r="B58" t="s">
-        <v>244</v>
+        <v>282</v>
       </c>
       <c r="C58" t="s">
-        <v>300</v>
+        <v>283</v>
       </c>
       <c r="D58" t="s">
-        <v>140</v>
+        <v>284</v>
       </c>
       <c r="E58" t="s">
-        <v>307</v>
+        <v>364</v>
       </c>
       <c r="F58" t="s">
-        <v>308</v>
+        <v>285</v>
       </c>
       <c r="G58" t="s">
         <v>11</v>
       </c>
       <c r="H58" t="s">
-        <v>231</v>
+        <v>276</v>
       </c>
       <c r="I58" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9">
+        <v>178</v>
+      </c>
+      <c r="J58" t="s">
+        <v>306</v>
+      </c>
+      <c r="K58" t="s">
+        <v>340</v>
+      </c>
+      <c r="L58" s="5" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12">
       <c r="A59" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B59" t="s">
-        <v>309</v>
+        <v>234</v>
       </c>
       <c r="C59" t="s">
-        <v>310</v>
+        <v>286</v>
       </c>
       <c r="D59" t="s">
-        <v>311</v>
+        <v>287</v>
       </c>
       <c r="E59" t="s">
-        <v>312</v>
+        <v>288</v>
       </c>
       <c r="F59" t="s">
-        <v>313</v>
+        <v>289</v>
       </c>
       <c r="G59" t="s">
         <v>11</v>
       </c>
       <c r="H59" t="s">
-        <v>297</v>
+        <v>276</v>
       </c>
       <c r="I59" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9">
+        <v>47</v>
+      </c>
+      <c r="J59" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12">
       <c r="A60" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B60" t="s">
-        <v>245</v>
+        <v>290</v>
       </c>
       <c r="C60" t="s">
-        <v>314</v>
+        <v>291</v>
       </c>
       <c r="D60" t="s">
-        <v>315</v>
+        <v>240</v>
       </c>
       <c r="E60" t="s">
-        <v>316</v>
+        <v>292</v>
       </c>
       <c r="F60" t="s">
-        <v>317</v>
+        <v>293</v>
       </c>
       <c r="G60" t="s">
         <v>11</v>
       </c>
       <c r="H60" t="s">
+        <v>276</v>
+      </c>
+      <c r="I60" t="s">
+        <v>178</v>
+      </c>
+      <c r="J60" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12">
+      <c r="A61" t="s">
+        <v>334</v>
+      </c>
+      <c r="B61" t="s">
+        <v>294</v>
+      </c>
+      <c r="C61" t="s">
+        <v>295</v>
+      </c>
+      <c r="D61" t="s">
+        <v>296</v>
+      </c>
+      <c r="E61" t="s">
         <v>297</v>
       </c>
-      <c r="I60" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9">
-      <c r="A61" t="s">
-        <v>333</v>
-      </c>
-      <c r="B61" t="s">
-        <v>318</v>
-      </c>
-      <c r="C61" t="s">
-        <v>319</v>
-      </c>
-      <c r="D61" t="s">
-        <v>251</v>
-      </c>
-      <c r="E61" t="s">
-        <v>320</v>
-      </c>
       <c r="F61" t="s">
-        <v>321</v>
+        <v>298</v>
       </c>
       <c r="G61" t="s">
         <v>11</v>
       </c>
       <c r="H61" t="s">
-        <v>297</v>
+        <v>276</v>
       </c>
       <c r="I61" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="62" spans="1:9">
+        <v>178</v>
+      </c>
+      <c r="J61" t="s">
+        <v>306</v>
+      </c>
+      <c r="K61" t="s">
+        <v>336</v>
+      </c>
+      <c r="L61" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12">
       <c r="A62" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B62" t="s">
-        <v>322</v>
+        <v>299</v>
       </c>
       <c r="C62" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="D62" t="s">
-        <v>324</v>
+        <v>210</v>
       </c>
       <c r="E62" t="s">
-        <v>325</v>
+        <v>301</v>
       </c>
       <c r="F62" t="s">
-        <v>326</v>
+        <v>302</v>
       </c>
       <c r="G62" t="s">
         <v>11</v>
       </c>
       <c r="H62" t="s">
-        <v>297</v>
+        <v>276</v>
       </c>
       <c r="I62" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9">
-      <c r="A63" t="s">
-        <v>335</v>
-      </c>
-      <c r="B63" t="s">
-        <v>327</v>
-      </c>
-      <c r="C63" t="s">
-        <v>328</v>
-      </c>
-      <c r="D63" t="s">
-        <v>220</v>
-      </c>
-      <c r="E63" t="s">
-        <v>329</v>
-      </c>
-      <c r="F63" t="s">
-        <v>330</v>
-      </c>
-      <c r="G63" t="s">
-        <v>11</v>
-      </c>
-      <c r="H63" t="s">
-        <v>297</v>
-      </c>
-      <c r="I63" t="s">
-        <v>188</v>
+        <v>178</v>
+      </c>
+      <c r="J62" t="s">
+        <v>305</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>